<commit_message>
chore: sync current working version before next phase
</commit_message>
<xml_diff>
--- a/runtime/apps/wechat_ai_customer_service/test_artifacts/file_transfer_smoke_customer_leads.xlsx
+++ b/runtime/apps/wechat_ai_customer_service/test_artifacts/file_transfer_smoke_customer_leads.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -572,9 +572,6 @@
           <t>2台</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>买7台冰箱能按20台价格吗？
@@ -587,6 +584,274 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-05-08T06:09:42</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>文件传输助手</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>m-discount,m-data</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>林晓晨</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>13800138001</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>上海市浦东新区张江路88号</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>商用冰箱</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2台</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>买7台冰箱能按20台价格吗？
+客户资料
+姓名：林晓晨
+电话：13800138001
+地址：上海市浦东新区张江路88号
+产品：商用冰箱
+数量：2台</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-05-08T06:10:11</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>文件传输助手</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>m-discount,m-data</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>林晓晨</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>13800138001</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>上海市浦东新区张江路88号</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>商用冰箱</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2台</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>买7台冰箱能按20台价格吗？
+客户资料
+姓名：林晓晨
+电话：13800138001
+地址：上海市浦东新区张江路88号
+产品：商用冰箱
+数量：2台</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-05-08T06:10:22</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>文件传输助手</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>m-discount,m-data</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>林晓晨</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>13800138001</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>上海市浦东新区张江路88号</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>商用冰箱</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2台</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>买7台冰箱能按20台价格吗？
+客户资料
+姓名：林晓晨
+电话：13800138001
+地址：上海市浦东新区张江路88号
+产品：商用冰箱
+数量：2台</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-05-08T06:10:34</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>文件传输助手</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>m-discount,m-data</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>林晓晨</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>13800138001</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>上海市浦东新区张江路88号</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>商用冰箱</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2台</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>买7台冰箱能按20台价格吗？
+客户资料
+姓名：林晓晨
+电话：13800138001
+地址：上海市浦东新区张江路88号
+产品：商用冰箱
+数量：2台</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-05-08T06:18:00</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>文件传输助手</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>m-discount,m-data</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>林晓晨</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>13800138001</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>上海市浦东新区张江路88号</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>商用冰箱</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2台</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>买7台冰箱能按20台价格吗？
+客户资料
+姓名：林晓晨
+电话：13800138001
+地址：上海市浦东新区张江路88号
+产品：商用冰箱
+数量：2台</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: publish current omniauto test snapshot
Publish the current local OmniAuto snapshot on top of the latest GitHub master.
Includes the chejin test account data, local auth/VPS simulation state, tenant RAG/raw knowledge data, and current WeChat customer-service code.
Ephemeral logs, lock files, pid files, and migration backup folders are intentionally left out of the published tree.
</commit_message>
<xml_diff>
--- a/runtime/apps/wechat_ai_customer_service/test_artifacts/file_transfer_smoke_customer_leads.xlsx
+++ b/runtime/apps/wechat_ai_customer_service/test_artifacts/file_transfer_smoke_customer_leads.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="客户线索" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="客户线索" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -837,9 +837,6 @@
           <t>2台</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
           <t>买7台冰箱能按20台价格吗？
@@ -852,6 +849,274 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-05-16T00:27:19</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>文件传输助手</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>m-discount,m-data</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>林晓晨</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>13800138001</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>上海市浦东新区张江路88号</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>商用冰箱</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2台</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>买7台冰箱能按20台价格吗？
+客户资料
+姓名：林晓晨
+电话：13800138001
+地址：上海市浦东新区张江路88号
+产品：商用冰箱
+数量：2台</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-05-16T00:30:10</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>文件传输助手</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>m-discount,m-data</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>林晓晨</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>13800138001</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>上海市浦东新区张江路88号</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>商用冰箱</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2台</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>买7台冰箱能按20台价格吗？
+客户资料
+姓名：林晓晨
+电话：13800138001
+地址：上海市浦东新区张江路88号
+产品：商用冰箱
+数量：2台</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-05-16T00:59:18</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>文件传输助手</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>m-discount,m-data</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>林晓晨</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>13800138001</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>上海市浦东新区张江路88号</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>商用冰箱</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2台</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>买7台冰箱能按20台价格吗？
+客户资料
+姓名：林晓晨
+电话：13800138001
+地址：上海市浦东新区张江路88号
+产品：商用冰箱
+数量：2台</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-05-16T02:35:04</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>文件传输助手</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>m-discount,m-data</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>林晓晨</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>13800138001</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>上海市浦东新区张江路88号</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>商用冰箱</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2台</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>买7台冰箱能按20台价格吗？
+客户资料
+姓名：林晓晨
+电话：13800138001
+地址：上海市浦东新区张江路88号
+产品：商用冰箱
+数量：2台</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-05-16T02:39:48</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>文件传输助手</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>m-discount,m-data</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>林晓晨</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>13800138001</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>上海市浦东新区张江路88号</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>商用冰箱</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2台</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>买7台冰箱能按20台价格吗？
+客户资料
+姓名：林晓晨
+电话：13800138001
+地址：上海市浦东新区张江路88号
+产品：商用冰箱
+数量：2台</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>